<commit_message>
added updates to the observation on the images generated after making changes to the threshold
</commit_message>
<xml_diff>
--- a/simulation_images_size_VS_concentrations.xlsx
+++ b/simulation_images_size_VS_concentrations.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="generated_image" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Row_encoder_5" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Row_encoder_5_on_updated_images" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="6">
   <si>
     <t xml:space="preserve">Concentration\MeanSize(um)</t>
   </si>
@@ -50,7 +51,7 @@
     <numFmt numFmtId="165" formatCode="0.E+00"/>
     <numFmt numFmtId="166" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -71,11 +72,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -134,48 +130,52 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -202,9 +202,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>88200</xdr:colOff>
+      <xdr:colOff>87840</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>4818600</xdr:rowOff>
+      <xdr:rowOff>4818240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -219,7 +219,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1721880" y="653400"/>
-          <a:ext cx="1315440" cy="4812840"/>
+          <a:ext cx="1315080" cy="4812480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -240,9 +240,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>4680</xdr:colOff>
+      <xdr:colOff>4320</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>3240</xdr:rowOff>
+      <xdr:rowOff>2880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -257,7 +257,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2953800" y="653040"/>
-          <a:ext cx="1233720" cy="4865040"/>
+          <a:ext cx="1233360" cy="4864680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -278,9 +278,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>9360</xdr:colOff>
+      <xdr:colOff>9000</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>1800</xdr:rowOff>
+      <xdr:rowOff>1440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -295,7 +295,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4265640" y="651240"/>
-          <a:ext cx="1160280" cy="4865400"/>
+          <a:ext cx="1159920" cy="4865040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -316,9 +316,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>11160</xdr:colOff>
+      <xdr:colOff>10800</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>4866840</xdr:rowOff>
+      <xdr:rowOff>4866480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -333,7 +333,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5422320" y="651240"/>
-          <a:ext cx="1239120" cy="4863240"/>
+          <a:ext cx="1238760" cy="4862880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -353,10 +353,10 @@
       <xdr:rowOff>7200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>720</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1433520</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>3240</xdr:rowOff>
+      <xdr:rowOff>2880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -371,7 +371,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6747480" y="654840"/>
-          <a:ext cx="1336680" cy="4863240"/>
+          <a:ext cx="1336320" cy="4862880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -392,9 +392,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>17280</xdr:colOff>
+      <xdr:colOff>16920</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>4834440</xdr:rowOff>
+      <xdr:rowOff>4834080</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -409,7 +409,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1724760" y="5533200"/>
-          <a:ext cx="1241640" cy="4816080"/>
+          <a:ext cx="1241280" cy="4815720"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -430,9 +430,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>71280</xdr:colOff>
+      <xdr:colOff>70920</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>4861080</xdr:rowOff>
+      <xdr:rowOff>4860720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -447,7 +447,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3042000" y="5507640"/>
-          <a:ext cx="1212120" cy="4868280"/>
+          <a:ext cx="1211760" cy="4867920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -468,9 +468,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>78840</xdr:colOff>
+      <xdr:colOff>78480</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>4838040</xdr:rowOff>
+      <xdr:rowOff>4837680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -485,7 +485,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4284000" y="5507640"/>
-          <a:ext cx="1211400" cy="4845240"/>
+          <a:ext cx="1211040" cy="4844880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -506,9 +506,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>88200</xdr:colOff>
+      <xdr:colOff>87840</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>4861800</xdr:rowOff>
+      <xdr:rowOff>4861440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -523,7 +523,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5417280" y="5511240"/>
-          <a:ext cx="1321200" cy="4865400"/>
+          <a:ext cx="1320840" cy="4865040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -544,9 +544,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>9000</xdr:colOff>
+      <xdr:colOff>8640</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>4837320</xdr:rowOff>
+      <xdr:rowOff>4836960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -561,7 +561,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6657840" y="5500440"/>
-          <a:ext cx="1434600" cy="4851720"/>
+          <a:ext cx="1434240" cy="4851360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -582,9 +582,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>69480</xdr:colOff>
+      <xdr:colOff>69120</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>4808520</xdr:rowOff>
+      <xdr:rowOff>4808160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -599,7 +599,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1849680" y="10382400"/>
-          <a:ext cx="1168920" cy="4808520"/>
+          <a:ext cx="1168560" cy="4808160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -620,9 +620,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>98280</xdr:colOff>
+      <xdr:colOff>97920</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>41400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -637,7 +637,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3038400" y="10387440"/>
-          <a:ext cx="1242720" cy="4903920"/>
+          <a:ext cx="1242360" cy="4903560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -658,9 +658,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>20880</xdr:colOff>
+      <xdr:colOff>20520</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>6480</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -675,7 +675,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4194720" y="10382400"/>
-          <a:ext cx="1242720" cy="4873680"/>
+          <a:ext cx="1242360" cy="4873320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -696,9 +696,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>146520</xdr:colOff>
+      <xdr:colOff>146160</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -713,7 +713,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5449680" y="10382400"/>
-          <a:ext cx="1347120" cy="4889520"/>
+          <a:ext cx="1346760" cy="4889160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -734,9 +734,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>307800</xdr:colOff>
+      <xdr:colOff>307440</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>11520</xdr:rowOff>
+      <xdr:rowOff>11160</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -751,7 +751,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6795720" y="10382400"/>
-          <a:ext cx="1595520" cy="4878720"/>
+          <a:ext cx="1595160" cy="4878360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -772,9 +772,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>88200</xdr:colOff>
+      <xdr:colOff>87840</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>4835160</xdr:rowOff>
+      <xdr:rowOff>4834800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -789,7 +789,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1718640" y="15227280"/>
-          <a:ext cx="1318680" cy="4857480"/>
+          <a:ext cx="1318320" cy="4857120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -810,9 +810,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1080</xdr:colOff>
+      <xdr:colOff>720</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>32760</xdr:rowOff>
+      <xdr:rowOff>32400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -827,7 +827,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2958120" y="15249600"/>
-          <a:ext cx="1225800" cy="4899960"/>
+          <a:ext cx="1225440" cy="4899600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -848,9 +848,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>97560</xdr:colOff>
+      <xdr:colOff>97200</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>4858560</xdr:rowOff>
+      <xdr:rowOff>4858200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -865,7 +865,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4192920" y="15240240"/>
-          <a:ext cx="1321200" cy="4867920"/>
+          <a:ext cx="1320840" cy="4867560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -886,9 +886,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>156960</xdr:colOff>
+      <xdr:colOff>156600</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>28800</xdr:rowOff>
+      <xdr:rowOff>28440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -903,7 +903,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5468400" y="15256080"/>
-          <a:ext cx="1338840" cy="4889520"/>
+          <a:ext cx="1338480" cy="4889160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -924,9 +924,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>302400</xdr:colOff>
+      <xdr:colOff>302040</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>18000</xdr:rowOff>
+      <xdr:rowOff>17640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -941,7 +941,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6820920" y="15256080"/>
-          <a:ext cx="1564920" cy="4878720"/>
+          <a:ext cx="1564560" cy="4878360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -962,9 +962,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>85320</xdr:colOff>
+      <xdr:colOff>84960</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>4848120</xdr:rowOff>
+      <xdr:rowOff>4847760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -979,7 +979,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1722600" y="20107440"/>
-          <a:ext cx="1311840" cy="4857480"/>
+          <a:ext cx="1311480" cy="4857120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1000,9 +1000,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2520</xdr:colOff>
+      <xdr:colOff>2160</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>26280</xdr:rowOff>
+      <xdr:rowOff>25920</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1017,7 +1017,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2961360" y="20107440"/>
-          <a:ext cx="1224000" cy="4902840"/>
+          <a:ext cx="1223640" cy="4902480"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1038,9 +1038,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>98640</xdr:colOff>
+      <xdr:colOff>98280</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>6480</xdr:rowOff>
+      <xdr:rowOff>6120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1055,7 +1055,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4191480" y="20118960"/>
-          <a:ext cx="1323720" cy="4871520"/>
+          <a:ext cx="1323360" cy="4871160"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1076,9 +1076,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>92160</xdr:colOff>
+      <xdr:colOff>91800</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>4827240</xdr:rowOff>
+      <xdr:rowOff>4826880</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1093,7 +1093,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5506200" y="20107440"/>
-          <a:ext cx="1236240" cy="4836600"/>
+          <a:ext cx="1235880" cy="4836240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1114,9 +1114,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>2520</xdr:colOff>
+      <xdr:colOff>2160</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>4820040</xdr:rowOff>
+      <xdr:rowOff>4819680</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1131,7 +1131,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6667200" y="20058120"/>
-          <a:ext cx="1418760" cy="4878720"/>
+          <a:ext cx="1418400" cy="4878360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1152,9 +1152,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>64440</xdr:colOff>
+      <xdr:colOff>64080</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>2880</xdr:rowOff>
+      <xdr:rowOff>2520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1169,7 +1169,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="1837080" y="24996600"/>
-          <a:ext cx="1176480" cy="4857480"/>
+          <a:ext cx="1176120" cy="4857120"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1190,9 +1190,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>81720</xdr:colOff>
+      <xdr:colOff>81360</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>4854960</xdr:rowOff>
+      <xdr:rowOff>4854600</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1207,7 +1207,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3039120" y="24996600"/>
-          <a:ext cx="1225440" cy="4842360"/>
+          <a:ext cx="1225080" cy="4842000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1228,9 +1228,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1233360</xdr:colOff>
+      <xdr:colOff>1233000</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>4862160</xdr:rowOff>
+      <xdr:rowOff>4861800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1245,7 +1245,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4273560" y="24989760"/>
-          <a:ext cx="1142640" cy="4856400"/>
+          <a:ext cx="1142280" cy="4856040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1266,9 +1266,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>1234080</xdr:colOff>
+      <xdr:colOff>1233720</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>4862160</xdr:rowOff>
+      <xdr:rowOff>4861800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1283,7 +1283,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="5512680" y="24977880"/>
-          <a:ext cx="1137960" cy="4868280"/>
+          <a:ext cx="1137600" cy="4867920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1304,9 +1304,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>6480</xdr:colOff>
+      <xdr:colOff>6120</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>4862160</xdr:rowOff>
+      <xdr:rowOff>4861800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1321,7 +1321,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6660720" y="24977880"/>
-          <a:ext cx="1429200" cy="4868280"/>
+          <a:ext cx="1428840" cy="4867920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1450,122 +1450,122 @@
   <dimension ref="A2:F12"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="17.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="17.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.33"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="2"/>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="5" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="6" t="n">
         <v>500000000</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="6" t="n">
         <v>400000000</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="6" t="n">
         <v>300000000</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="6" t="n">
         <v>200000000</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="6" t="n">
         <v>100000000</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="6" t="n">
         <v>50000000</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="2"/>
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="2"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1587,311 +1587,649 @@
   <dimension ref="A5:F29"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.45"/>
   </cols>
   <sheetData>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="10" t="n">
         <f aca="false">generated_image!A5</f>
         <v>500000000</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>67836</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <v>51184</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <v>51162</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <v>72908</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10" t="n">
+      <c r="A9" s="10"/>
+      <c r="B9" s="11" t="n">
         <f aca="false">1-B8/C29</f>
         <v>0.275691691691692</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <f aca="false">1-C8/C29</f>
         <v>0.453490824157491</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">1-D8/C29</f>
         <v>0.453725725725726</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="11" t="n">
         <f aca="false">1-E8/C29</f>
         <v>0.221536202869536</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
+      <c r="A10" s="10" t="n">
         <f aca="false">generated_image!A6</f>
         <v>400000000</v>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="9" t="n">
         <v>56722</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="9" t="n">
         <v>38314</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <v>42758</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="9" t="n">
         <v>59744</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="10" t="n">
+      <c r="A11" s="10"/>
+      <c r="B11" s="11" t="n">
         <f aca="false">1-B10/C29</f>
         <v>0.39435969302636</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="11" t="n">
         <f aca="false">1-C10/C29</f>
         <v>0.590908241574908</v>
       </c>
-      <c r="D11" s="10" t="n">
+      <c r="D11" s="11" t="n">
         <f aca="false">1-D10/C29</f>
         <v>0.543458124791458</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="11" t="n">
         <f aca="false">1-E10/C29</f>
         <v>0.362092759426093</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="n">
+      <c r="A12" s="10" t="n">
         <f aca="false">generated_image!A7</f>
         <v>300000000</v>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="9" t="n">
         <v>48036</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="9" t="n">
         <v>25192</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="9" t="n">
         <v>26578</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="9" t="n">
         <v>52774</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="10" t="n">
+      <c r="A13" s="10"/>
+      <c r="B13" s="11" t="n">
         <f aca="false">1-B12/C29</f>
         <v>0.487103103103103</v>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="11" t="n">
         <f aca="false">1-C12/C29</f>
         <v>0.731016349683016</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <f aca="false">1-D12/C29</f>
         <v>0.716217550884218</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="11" t="n">
         <f aca="false">1-E12/C29</f>
         <v>0.436513847180514</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
+      <c r="A14" s="10" t="n">
         <f aca="false">generated_image!A8</f>
         <v>200000000</v>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>28362</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="9" t="n">
         <v>15682</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="9" t="n">
         <v>17966</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="9" t="n">
         <v>30324</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10" t="n">
+      <c r="A15" s="10"/>
+      <c r="B15" s="11" t="n">
         <f aca="false">1-B14/C29</f>
         <v>0.697169169169169</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="11" t="n">
         <f aca="false">1-C14/C29</f>
         <v>0.832557891224558</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <f aca="false">1-D14/C29</f>
         <v>0.808170837504171</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="11" t="n">
         <f aca="false">1-E14/C29</f>
         <v>0.67622022022022</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="n">
+      <c r="A16" s="10" t="n">
         <f aca="false">generated_image!A9</f>
         <v>100000000</v>
       </c>
-      <c r="B16" s="8" t="n">
+      <c r="B16" s="9" t="n">
         <v>8826</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="9" t="n">
         <v>6662</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="9" t="n">
         <v>6114</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="9" t="n">
         <v>12482</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10" t="n">
+      <c r="A17" s="10"/>
+      <c r="B17" s="11" t="n">
         <f aca="false">1-B16/C29</f>
         <v>0.905761761761762</v>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="11" t="n">
         <f aca="false">1-C16/C29</f>
         <v>0.928867534200868</v>
       </c>
-      <c r="D17" s="10" t="n">
+      <c r="D17" s="11" t="n">
         <f aca="false">1-D16/C29</f>
         <v>0.934718718718719</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="11" t="n">
         <f aca="false">1-E16/C29</f>
         <v>0.866725392058726</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="n">
+      <c r="A18" s="10" t="n">
         <f aca="false">generated_image!A10</f>
         <v>50000000</v>
       </c>
-      <c r="B18" s="8" t="n">
+      <c r="B18" s="9" t="n">
         <v>4684</v>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="9" t="n">
         <v>2648</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="9" t="n">
         <v>2942</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="9" t="n">
         <v>8384</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10" t="n">
+      <c r="A19" s="10"/>
+      <c r="B19" s="11" t="n">
         <f aca="false">1-B18/C29</f>
         <v>0.949987320653987</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="11" t="n">
         <f aca="false">1-C18/C29</f>
         <v>0.971726393059726</v>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">1-D18/C29</f>
         <v>0.968587253920587</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="11" t="n">
         <f aca="false">1-E18/C29</f>
         <v>0.910481147814481</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="9" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C29" s="0" t="n">
+      <c r="C29" s="1" t="n">
+        <f aca="false">999*250*3/8</f>
+        <v>93656.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A5:F29"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.45"/>
+  </cols>
+  <sheetData>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="n">
+        <f aca="false">generated_image!A5</f>
+        <v>500000000</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>14600</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>7060</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>10038</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>27584</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10"/>
+      <c r="B9" s="11" t="n">
+        <f aca="false">1-B8/C29</f>
+        <v>0.844110777444111</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <f aca="false">1-C8/C29</f>
+        <v>0.924617951284618</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <f aca="false">1-D8/C29</f>
+        <v>0.892820820820821</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <f aca="false">1-E8/C29</f>
+        <v>0.705476142809476</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="n">
+        <f aca="false">generated_image!A6</f>
+        <v>400000000</v>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>10702</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>5208</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>8060</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>20638</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10"/>
+      <c r="B11" s="11" t="n">
+        <f aca="false">1-B10/C29</f>
+        <v>0.885731064397731</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <f aca="false">1-C10/C29</f>
+        <v>0.944392392392392</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <f aca="false">1-D10/C29</f>
+        <v>0.913940607273941</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <f aca="false">1-E10/C29</f>
+        <v>0.779640974307641</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
+        <f aca="false">generated_image!A7</f>
+        <v>300000000</v>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>7210</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>2964</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>4152</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>14522</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10"/>
+      <c r="B13" s="11" t="n">
+        <f aca="false">1-B12/C29</f>
+        <v>0.923016349683016</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <f aca="false">1-C12/C29</f>
+        <v>0.968352352352352</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <f aca="false">1-D12/C29</f>
+        <v>0.955667667667668</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <f aca="false">1-E12/C29</f>
+        <v>0.844943610276944</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
+        <f aca="false">generated_image!A8</f>
+        <v>200000000</v>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>3540</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>2406</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>3076</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>9250</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10"/>
+      <c r="B15" s="11" t="n">
+        <f aca="false">1-B14/C29</f>
+        <v>0.962202202202202</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <f aca="false">1-C14/C29</f>
+        <v>0.97431031031031</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <f aca="false">1-D14/C29</f>
+        <v>0.967156489823157</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <f aca="false">1-E14/C29</f>
+        <v>0.901234567901235</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
+        <f aca="false">generated_image!A9</f>
+        <v>100000000</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>1330</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>860</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>1346</v>
+      </c>
+      <c r="E16" s="9" t="n">
+        <v>3814</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10"/>
+      <c r="B17" s="11" t="n">
+        <f aca="false">1-B16/C29</f>
+        <v>0.985799132465799</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <f aca="false">1-C16/C29</f>
+        <v>0.990817484150818</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <f aca="false">1-D16/C29</f>
+        <v>0.985628294961628</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <f aca="false">1-E16/C29</f>
+        <v>0.959276609943277</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
+        <f aca="false">generated_image!A10</f>
+        <v>50000000</v>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>746</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>286</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>718</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>3146</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10"/>
+      <c r="B19" s="11" t="n">
+        <f aca="false">1-B18/C29</f>
+        <v>0.992034701368035</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <f aca="false">1-C18/C29</f>
+        <v>0.996946279612946</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <f aca="false">1-D18/C29</f>
+        <v>0.992333667000334</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <f aca="false">1-E18/C29</f>
+        <v>0.966409075742409</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="1" t="n">
         <f aca="false">999*250*3/8</f>
         <v>93656.25</v>
       </c>

</xml_diff>

<commit_message>
added updated images to the xlsx file
</commit_message>
<xml_diff>
--- a/simulation_images_size_VS_concentrations.xlsx
+++ b/simulation_images_size_VS_concentrations.xlsx
@@ -1,19 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shouyuxie/MD_log/reImplement_Compress/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF1AA4A-B2D7-6E4D-9E94-65E0B88F14A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="generated_image" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Row_encoder_5" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Row_encoder_5_on_updated_images" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="generated_image" sheetId="1" r:id="rId1"/>
+    <sheet name="Row_encoder_5" sheetId="2" r:id="rId2"/>
+    <sheet name="generated_image_new_theta" sheetId="4" r:id="rId3"/>
+    <sheet name="Row_encoder_5_on_updated_images" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1"/>
     </ext>
@@ -21,57 +38,352 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="30">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="9"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="10"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="11"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="12"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="13"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="14"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="15"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="16"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="17"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="18"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="19"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="20"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="21"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="22"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="23"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="24"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="25"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="26"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="27"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="28"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="29"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="30">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
+    </bk>
+    <bk>
+      <rc t="1" v="8"/>
+    </bk>
+    <bk>
+      <rc t="1" v="9"/>
+    </bk>
+    <bk>
+      <rc t="1" v="10"/>
+    </bk>
+    <bk>
+      <rc t="1" v="11"/>
+    </bk>
+    <bk>
+      <rc t="1" v="12"/>
+    </bk>
+    <bk>
+      <rc t="1" v="13"/>
+    </bk>
+    <bk>
+      <rc t="1" v="14"/>
+    </bk>
+    <bk>
+      <rc t="1" v="15"/>
+    </bk>
+    <bk>
+      <rc t="1" v="16"/>
+    </bk>
+    <bk>
+      <rc t="1" v="17"/>
+    </bk>
+    <bk>
+      <rc t="1" v="18"/>
+    </bk>
+    <bk>
+      <rc t="1" v="19"/>
+    </bk>
+    <bk>
+      <rc t="1" v="20"/>
+    </bk>
+    <bk>
+      <rc t="1" v="21"/>
+    </bk>
+    <bk>
+      <rc t="1" v="22"/>
+    </bk>
+    <bk>
+      <rc t="1" v="23"/>
+    </bk>
+    <bk>
+      <rc t="1" v="24"/>
+    </bk>
+    <bk>
+      <rc t="1" v="25"/>
+    </bk>
+    <bk>
+      <rc t="1" v="26"/>
+    </bk>
+    <bk>
+      <rc t="1" v="27"/>
+    </bk>
+    <bk>
+      <rc t="1" v="28"/>
+    </bk>
+    <bk>
+      <rc t="1" v="29"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="6">
   <si>
-    <t xml:space="preserve">Concentration\MeanSize(um)</t>
+    <t>Concentration\MeanSize(um)</t>
   </si>
   <si>
-    <t xml:space="preserve">Total compressed size (byte)</t>
+    <t>Total compressed size (byte)</t>
   </si>
   <si>
-    <t xml:space="preserve">Mean size(um)</t>
+    <t>Mean size(um)</t>
   </si>
   <si>
-    <t xml:space="preserve">Concentration</t>
+    <t>Concentration</t>
   </si>
   <si>
-    <t xml:space="preserve">n/a</t>
+    <t>n/a</t>
   </si>
   <si>
-    <t xml:space="preserve">Raw size (byte)</t>
+    <t>Raw size (byte)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.E+00"/>
-    <numFmt numFmtId="166" formatCode="0.00%"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.E+00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -83,116 +395,87 @@
     </fill>
   </fills>
   <borders count="3">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="12">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -208,12 +491,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="Image 1" descr=""/>
+        <xdr:cNvPr id="2" name="Image 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:srcRect l="24685" t="0" r="20638" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:srcRect l="24685" r="20638"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -246,12 +535,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 2" descr=""/>
+        <xdr:cNvPr id="3" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:srcRect l="24661" t="0" r="20441" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:srcRect l="24661" r="20441"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -284,12 +579,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 3" descr=""/>
+        <xdr:cNvPr id="4" name="Image 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:srcRect l="24031" t="0" r="19906" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:srcRect l="24031" r="19906"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -322,12 +623,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 4" descr=""/>
+        <xdr:cNvPr id="5" name="Image 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:srcRect l="24591" t="0" r="20244" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:srcRect l="24591" r="20244"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -360,12 +667,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 5" descr=""/>
+        <xdr:cNvPr id="6" name="Image 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:srcRect l="28937" t="0" r="7157" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:srcRect l="28937" r="7157"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -398,12 +711,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 6" descr=""/>
+        <xdr:cNvPr id="7" name="Image 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId6"/>
-        <a:srcRect l="23976" t="0" r="20244" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:srcRect l="23976" r="20244"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -436,12 +755,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 7" descr=""/>
+        <xdr:cNvPr id="8" name="Image 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId7"/>
-        <a:srcRect l="24882" t="0" r="21126" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:srcRect l="24882" r="21126"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -474,12 +799,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 8" descr=""/>
+        <xdr:cNvPr id="9" name="Image 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId8"/>
-        <a:srcRect l="24732" t="0" r="21024" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:srcRect l="24732" r="21024"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -512,12 +843,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 9" descr=""/>
+        <xdr:cNvPr id="10" name="Image 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId9"/>
-        <a:srcRect l="24661" t="0" r="20976" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:srcRect l="24661" r="20976"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -550,12 +887,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 10" descr=""/>
+        <xdr:cNvPr id="11" name="Image 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId10"/>
-        <a:srcRect l="28567" t="0" r="7449" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:srcRect l="28567" r="7449"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -588,12 +931,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 11" descr=""/>
+        <xdr:cNvPr id="12" name="Image 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId11"/>
-        <a:srcRect l="24732" t="0" r="20976" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:srcRect l="24732" r="20976"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -626,12 +975,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 12" descr=""/>
+        <xdr:cNvPr id="13" name="Image 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId12"/>
-        <a:srcRect l="24906" t="0" r="20732" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:srcRect l="24906" r="20732"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -664,12 +1019,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 13" descr=""/>
+        <xdr:cNvPr id="14" name="Image 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId13"/>
-        <a:srcRect l="24709" t="0" r="21071" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:srcRect l="24709" r="21071"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -702,12 +1063,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 14" descr=""/>
+        <xdr:cNvPr id="15" name="Image 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId14"/>
-        <a:srcRect l="24417" t="0" r="20780" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
+        <a:srcRect l="24417" r="20780"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -740,12 +1107,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 15" descr=""/>
+        <xdr:cNvPr id="16" name="Image 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId15"/>
-        <a:srcRect l="28079" t="0" r="7157" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:srcRect l="28079" r="7157"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -778,12 +1151,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="Image 16" descr=""/>
+        <xdr:cNvPr id="17" name="Image 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId16"/>
-        <a:srcRect l="25008" t="0" r="20535" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:srcRect l="25008" r="20535"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -816,12 +1195,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="Image 17" descr=""/>
+        <xdr:cNvPr id="18" name="Image 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId17"/>
-        <a:srcRect l="25008" t="0" r="20780" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:srcRect l="25008" r="20780"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -854,12 +1239,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="Image 18" descr=""/>
+        <xdr:cNvPr id="19" name="Image 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId18"/>
-        <a:srcRect l="24787" t="0" r="21071" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:srcRect l="24787" r="21071"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -892,12 +1283,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Image 19" descr=""/>
+        <xdr:cNvPr id="20" name="Image 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000014000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId19"/>
-        <a:srcRect l="24787" t="0" r="20732" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:srcRect l="24787" r="20732"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -930,12 +1327,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="Image 20" descr=""/>
+        <xdr:cNvPr id="21" name="Image 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000015000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId20"/>
-        <a:srcRect l="28787" t="0" r="7646" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:srcRect l="28787" r="7646"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -968,12 +1371,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="20" name="Image 21" descr=""/>
+        <xdr:cNvPr id="22" name="Image 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000016000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId21"/>
-        <a:srcRect l="24906" t="0" r="20976" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:srcRect l="24906" r="20976"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1006,12 +1415,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="Image 22" descr=""/>
+        <xdr:cNvPr id="23" name="Image 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000017000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId22"/>
-        <a:srcRect l="24882" t="0" r="20976" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:srcRect l="24882" r="20976"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1044,12 +1459,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="22" name="Image 23" descr=""/>
+        <xdr:cNvPr id="24" name="Image 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000018000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId23"/>
-        <a:srcRect l="24906" t="0" r="21024" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:srcRect l="24906" r="21024"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1082,12 +1503,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Image 24" descr=""/>
+        <xdr:cNvPr id="25" name="Image 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000019000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId24"/>
-        <a:srcRect l="24858" t="0" r="20976" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:srcRect l="24858" r="20976"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1120,12 +1547,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="24" name="Image 25" descr=""/>
+        <xdr:cNvPr id="26" name="Image 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId25"/>
-        <a:srcRect l="28787" t="0" r="8331" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:srcRect l="28787" r="8331"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1158,12 +1591,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="Image 26" descr=""/>
+        <xdr:cNvPr id="27" name="Image 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId26"/>
-        <a:srcRect l="24929" t="0" r="20732" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:srcRect l="24929" r="20732"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1196,12 +1635,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="Image 27" descr=""/>
+        <xdr:cNvPr id="28" name="Image 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId27"/>
-        <a:srcRect l="25031" t="0" r="20780" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:srcRect l="25031" r="20780"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1234,12 +1679,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="27" name="Image 28" descr=""/>
+        <xdr:cNvPr id="29" name="Image 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId28"/>
-        <a:srcRect l="24953" t="0" r="20929" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <a:srcRect l="24953" r="20929"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1272,12 +1723,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="28" name="Image 29" descr=""/>
+        <xdr:cNvPr id="30" name="Image 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId29"/>
-        <a:srcRect l="25008" t="0" r="20827" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <a:srcRect l="25008" r="20827"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1310,12 +1767,18 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="29" name="Image 30" descr=""/>
+        <xdr:cNvPr id="31" name="Image 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00001F000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId30"/>
-        <a:srcRect l="28717" t="0" r="7504" b="0"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:srcRect l="28717" r="7504"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
@@ -1336,57 +1799,266 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="30">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>10</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>11</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>12</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>13</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>14</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>15</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>16</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>17</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>18</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>19</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>20</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>21</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>22</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>23</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>24</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>25</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>26</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>27</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>28</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>29</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+  <rel r:id="rId10"/>
+  <rel r:id="rId11"/>
+  <rel r:id="rId12"/>
+  <rel r:id="rId13"/>
+  <rel r:id="rId14"/>
+  <rel r:id="rId15"/>
+  <rel r:id="rId16"/>
+  <rel r:id="rId17"/>
+  <rel r:id="rId18"/>
+  <rel r:id="rId19"/>
+  <rel r:id="rId20"/>
+  <rel r:id="rId21"/>
+  <rel r:id="rId22"/>
+  <rel r:id="rId23"/>
+  <rel r:id="rId24"/>
+  <rel r:id="rId25"/>
+  <rel r:id="rId26"/>
+  <rel r:id="rId27"/>
+  <rel r:id="rId28"/>
+  <rel r:id="rId29"/>
+  <rel r:id="rId30"/>
+</richValueRels>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="LibreOffice">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Arial"/>
+        <a:ea typeface="DejaVu Sans"/>
+        <a:cs typeface="DejaVu Sans"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1439,139 +2111,137 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:F12"/>
-  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="17.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.33"/>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="2" max="5" width="17.5" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5">
         <v>30</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5">
         <v>20</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5">
         <v>10</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5">
         <v>5</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+    <row r="5" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="7">
         <v>500000000</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="7">
         <v>400000000</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="7">
         <v>300000000</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="4"/>
+    </row>
+    <row r="8" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="7">
         <v>200000000</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="3"/>
-    </row>
-    <row r="9" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="7">
         <v>100000000</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" customFormat="false" ht="383.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="7">
         <v>50000000</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="4"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="4"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
@@ -1580,337 +2250,333 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A5:F29"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.45"/>
+    <col min="1" max="1" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="7" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="7" t="s">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8">
         <v>30</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8">
         <v>20</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8">
         <v>10</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8">
         <v>5</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
-        <f aca="false">generated_image!A5</f>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A8" s="1">
+        <f>generated_image!A5</f>
         <v>500000000</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8">
         <v>67836</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="8">
         <v>51184</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="8">
         <v>51162</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="8">
         <v>72908</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11" t="n">
-        <f aca="false">1-B8/C29</f>
-        <v>0.275691691691692</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <f aca="false">1-C8/C29</f>
-        <v>0.453490824157491</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">1-D8/C29</f>
-        <v>0.453725725725726</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <f aca="false">1-E8/C29</f>
-        <v>0.221536202869536</v>
-      </c>
-      <c r="F9" s="9" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A9" s="1"/>
+      <c r="B9" s="9">
+        <f>1-B8/C29</f>
+        <v>0.27569169169169172</v>
+      </c>
+      <c r="C9" s="9">
+        <f>1-C8/C29</f>
+        <v>0.45349082415749087</v>
+      </c>
+      <c r="D9" s="9">
+        <f>1-D8/C29</f>
+        <v>0.45372572572572567</v>
+      </c>
+      <c r="E9" s="9">
+        <f>1-E8/C29</f>
+        <v>0.22153620286953624</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
-        <f aca="false">generated_image!A6</f>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A10" s="1">
+        <f>generated_image!A6</f>
         <v>400000000</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8">
         <v>56722</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="8">
         <v>38314</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="8">
         <v>42758</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="8">
         <v>59744</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11" t="n">
-        <f aca="false">1-B10/C29</f>
-        <v>0.39435969302636</v>
-      </c>
-      <c r="C11" s="11" t="n">
-        <f aca="false">1-C10/C29</f>
-        <v>0.590908241574908</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <f aca="false">1-D10/C29</f>
-        <v>0.543458124791458</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <f aca="false">1-E10/C29</f>
-        <v>0.362092759426093</v>
-      </c>
-      <c r="F11" s="9" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A11" s="1"/>
+      <c r="B11" s="9">
+        <f>1-B10/C29</f>
+        <v>0.39435969302635965</v>
+      </c>
+      <c r="C11" s="9">
+        <f>1-C10/C29</f>
+        <v>0.59090824157490829</v>
+      </c>
+      <c r="D11" s="9">
+        <f>1-D10/C29</f>
+        <v>0.54345812479145805</v>
+      </c>
+      <c r="E11" s="9">
+        <f>1-E10/C29</f>
+        <v>0.36209275942609276</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
-        <f aca="false">generated_image!A7</f>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A12" s="1">
+        <f>generated_image!A7</f>
         <v>300000000</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="8">
         <v>48036</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="8">
         <v>25192</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="8">
         <v>26578</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="8">
         <v>52774</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11" t="n">
-        <f aca="false">1-B12/C29</f>
-        <v>0.487103103103103</v>
-      </c>
-      <c r="C13" s="11" t="n">
-        <f aca="false">1-C12/C29</f>
-        <v>0.731016349683016</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <f aca="false">1-D12/C29</f>
-        <v>0.716217550884218</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <f aca="false">1-E12/C29</f>
-        <v>0.436513847180514</v>
-      </c>
-      <c r="F13" s="9" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A13" s="1"/>
+      <c r="B13" s="9">
+        <f>1-B12/C29</f>
+        <v>0.48710310310310312</v>
+      </c>
+      <c r="C13" s="9">
+        <f>1-C12/C29</f>
+        <v>0.73101634968301643</v>
+      </c>
+      <c r="D13" s="9">
+        <f>1-D12/C29</f>
+        <v>0.71621755088421757</v>
+      </c>
+      <c r="E13" s="9">
+        <f>1-E12/C29</f>
+        <v>0.43651384718051389</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
-        <f aca="false">generated_image!A8</f>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A14" s="1">
+        <f>generated_image!A8</f>
         <v>200000000</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8">
         <v>28362</v>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="8">
         <v>15682</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="8">
         <v>17966</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="8">
         <v>30324</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11" t="n">
-        <f aca="false">1-B14/C29</f>
-        <v>0.697169169169169</v>
-      </c>
-      <c r="C15" s="11" t="n">
-        <f aca="false">1-C14/C29</f>
-        <v>0.832557891224558</v>
-      </c>
-      <c r="D15" s="11" t="n">
-        <f aca="false">1-D14/C29</f>
-        <v>0.808170837504171</v>
-      </c>
-      <c r="E15" s="11" t="n">
-        <f aca="false">1-E14/C29</f>
-        <v>0.67622022022022</v>
-      </c>
-      <c r="F15" s="9" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A15" s="1"/>
+      <c r="B15" s="9">
+        <f>1-B14/C29</f>
+        <v>0.69716916916916916</v>
+      </c>
+      <c r="C15" s="9">
+        <f>1-C14/C29</f>
+        <v>0.83255789122455792</v>
+      </c>
+      <c r="D15" s="9">
+        <f>1-D14/C29</f>
+        <v>0.80817083750417085</v>
+      </c>
+      <c r="E15" s="9">
+        <f>1-E14/C29</f>
+        <v>0.67622022022022021</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
-        <f aca="false">generated_image!A9</f>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A16" s="1">
+        <f>generated_image!A9</f>
         <v>100000000</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="8">
         <v>8826</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="8">
         <v>6662</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="8">
         <v>6114</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="8">
         <v>12482</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11" t="n">
-        <f aca="false">1-B16/C29</f>
-        <v>0.905761761761762</v>
-      </c>
-      <c r="C17" s="11" t="n">
-        <f aca="false">1-C16/C29</f>
-        <v>0.928867534200868</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <f aca="false">1-D16/C29</f>
-        <v>0.934718718718719</v>
-      </c>
-      <c r="E17" s="11" t="n">
-        <f aca="false">1-E16/C29</f>
-        <v>0.866725392058726</v>
-      </c>
-      <c r="F17" s="9" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A17" s="1"/>
+      <c r="B17" s="9">
+        <f>1-B16/C29</f>
+        <v>0.90576176176176171</v>
+      </c>
+      <c r="C17" s="9">
+        <f>1-C16/C29</f>
+        <v>0.92886753420086754</v>
+      </c>
+      <c r="D17" s="9">
+        <f>1-D16/C29</f>
+        <v>0.9347187187187187</v>
+      </c>
+      <c r="E17" s="9">
+        <f>1-E16/C29</f>
+        <v>0.86672539205872545</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
-        <f aca="false">generated_image!A10</f>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A18" s="1">
+        <f>generated_image!A10</f>
         <v>50000000</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="8">
         <v>4684</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="8">
         <v>2648</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="8">
         <v>2942</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="8">
         <v>8384</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11" t="n">
-        <f aca="false">1-B18/C29</f>
-        <v>0.949987320653987</v>
-      </c>
-      <c r="C19" s="11" t="n">
-        <f aca="false">1-C18/C29</f>
-        <v>0.971726393059726</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <f aca="false">1-D18/C29</f>
-        <v>0.968587253920587</v>
-      </c>
-      <c r="E19" s="11" t="n">
-        <f aca="false">1-E18/C29</f>
-        <v>0.910481147814481</v>
-      </c>
-      <c r="F19" s="9" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A19" s="1"/>
+      <c r="B19" s="9">
+        <f>1-B18/C29</f>
+        <v>0.94998732065398728</v>
+      </c>
+      <c r="C19" s="9">
+        <f>1-C18/C29</f>
+        <v>0.97172639305972641</v>
+      </c>
+      <c r="D19" s="9">
+        <f>1-D18/C29</f>
+        <v>0.96858725392058731</v>
+      </c>
+      <c r="E19" s="9">
+        <f>1-E18/C29</f>
+        <v>0.9104811478144812</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="1" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B29" t="s">
         <v>5</v>
       </c>
-      <c r="C29" s="1" t="n">
-        <f aca="false">999*250*3/8</f>
+      <c r="C29">
+        <f>999*250*3/8</f>
         <v>93656.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A19"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
@@ -1918,337 +2584,525 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A5:F29"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EB660E2-51F1-3343-8122-78F07AEEE22A}">
+  <dimension ref="A2:F12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.45"/>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
+    <col min="2" max="5" width="17.5" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="7" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="5">
+        <v>30</v>
+      </c>
+      <c r="C4" s="5">
+        <v>20</v>
+      </c>
+      <c r="D4" s="5">
+        <v>10</v>
+      </c>
+      <c r="E4" s="5">
+        <v>5</v>
+      </c>
+      <c r="F4" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="7">
+        <v>500000000</v>
+      </c>
+      <c r="B5" s="3" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C5" s="3" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D5" s="3" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E5" s="3" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F5" s="4" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="7">
+        <v>400000000</v>
+      </c>
+      <c r="B6" s="3" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C6" s="3" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D6" s="3" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E6" s="3" t="e" vm="9">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F6" s="4" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="7">
+        <v>300000000</v>
+      </c>
+      <c r="B7" s="3" t="e" vm="11">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="3" t="e" vm="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D7" s="3" t="e" vm="13">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E7" s="3" t="e" vm="14">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F7" s="4" t="e" vm="15">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="7">
+        <v>200000000</v>
+      </c>
+      <c r="B8" s="3" t="e" vm="16">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C8" s="3" t="e" vm="17">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D8" s="3" t="e" vm="18">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E8" s="3" t="e" vm="19">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F8" s="4" t="e" vm="20">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="7">
+        <v>100000000</v>
+      </c>
+      <c r="B9" s="3" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C9" s="3" t="e" vm="22">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D9" s="3" t="e" vm="23">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E9" s="3" t="e" vm="24">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F9" s="4" t="e" vm="25">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="383.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="7">
+        <v>50000000</v>
+      </c>
+      <c r="B10" s="3" t="e" vm="26">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C10" s="3" t="e" vm="27">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D10" s="3" t="e" vm="28">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E10" s="3" t="e" vm="29">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F10" s="4" t="e" vm="30">
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="4"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A5:F29"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="13.1640625" customWidth="1"/>
+    <col min="2" max="2" width="12.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="7" t="s">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="8">
         <v>30</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8">
         <v>20</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8">
         <v>10</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8">
         <v>5</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
-        <f aca="false">generated_image!A5</f>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A8" s="1">
+        <f>generated_image!A5</f>
         <v>500000000</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8">
         <v>14600</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="8">
         <v>7060</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="8">
         <v>10038</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="8">
         <v>27584</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11" t="n">
-        <f aca="false">1-B8/C29</f>
-        <v>0.844110777444111</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <f aca="false">1-C8/C29</f>
-        <v>0.924617951284618</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">1-D8/C29</f>
-        <v>0.892820820820821</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <f aca="false">1-E8/C29</f>
-        <v>0.705476142809476</v>
-      </c>
-      <c r="F9" s="9" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A9" s="1"/>
+      <c r="B9" s="9">
+        <f>1-B8/C29</f>
+        <v>0.84411077744411078</v>
+      </c>
+      <c r="C9" s="9">
+        <f>1-C8/C29</f>
+        <v>0.92461795128461799</v>
+      </c>
+      <c r="D9" s="9">
+        <f>1-D8/C29</f>
+        <v>0.89282082082082082</v>
+      </c>
+      <c r="E9" s="9">
+        <f>1-E8/C29</f>
+        <v>0.70547614280947613</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
-        <f aca="false">generated_image!A6</f>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A10" s="1">
+        <f>generated_image!A6</f>
         <v>400000000</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8">
         <v>10702</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="8">
         <v>5208</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="8">
         <v>8060</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="8">
         <v>20638</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11" t="n">
-        <f aca="false">1-B10/C29</f>
-        <v>0.885731064397731</v>
-      </c>
-      <c r="C11" s="11" t="n">
-        <f aca="false">1-C10/C29</f>
-        <v>0.944392392392392</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <f aca="false">1-D10/C29</f>
-        <v>0.913940607273941</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <f aca="false">1-E10/C29</f>
-        <v>0.779640974307641</v>
-      </c>
-      <c r="F11" s="9" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A11" s="1"/>
+      <c r="B11" s="9">
+        <f>1-B10/C29</f>
+        <v>0.88573106439773108</v>
+      </c>
+      <c r="C11" s="9">
+        <f>1-C10/C29</f>
+        <v>0.94439239239239237</v>
+      </c>
+      <c r="D11" s="9">
+        <f>1-D10/C29</f>
+        <v>0.91394060727394066</v>
+      </c>
+      <c r="E11" s="9">
+        <f>1-E10/C29</f>
+        <v>0.77964097430764101</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
-        <f aca="false">generated_image!A7</f>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A12" s="1">
+        <f>generated_image!A7</f>
         <v>300000000</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="8">
         <v>7210</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="8">
         <v>2964</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="8">
         <v>4152</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="8">
         <v>14522</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11" t="n">
-        <f aca="false">1-B12/C29</f>
-        <v>0.923016349683016</v>
-      </c>
-      <c r="C13" s="11" t="n">
-        <f aca="false">1-C12/C29</f>
-        <v>0.968352352352352</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <f aca="false">1-D12/C29</f>
-        <v>0.955667667667668</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <f aca="false">1-E12/C29</f>
-        <v>0.844943610276944</v>
-      </c>
-      <c r="F13" s="9" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A13" s="1"/>
+      <c r="B13" s="9">
+        <f>1-B12/C29</f>
+        <v>0.92301634968301638</v>
+      </c>
+      <c r="C13" s="9">
+        <f>1-C12/C29</f>
+        <v>0.9683523523523524</v>
+      </c>
+      <c r="D13" s="9">
+        <f>1-D12/C29</f>
+        <v>0.95566766766766764</v>
+      </c>
+      <c r="E13" s="9">
+        <f>1-E12/C29</f>
+        <v>0.84494361027694365</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
-        <f aca="false">generated_image!A8</f>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A14" s="1">
+        <f>generated_image!A8</f>
         <v>200000000</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8">
         <v>3540</v>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="8">
         <v>2406</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="8">
         <v>3076</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="8">
         <v>9250</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11" t="n">
-        <f aca="false">1-B14/C29</f>
-        <v>0.962202202202202</v>
-      </c>
-      <c r="C15" s="11" t="n">
-        <f aca="false">1-C14/C29</f>
-        <v>0.97431031031031</v>
-      </c>
-      <c r="D15" s="11" t="n">
-        <f aca="false">1-D14/C29</f>
-        <v>0.967156489823157</v>
-      </c>
-      <c r="E15" s="11" t="n">
-        <f aca="false">1-E14/C29</f>
-        <v>0.901234567901235</v>
-      </c>
-      <c r="F15" s="9" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A15" s="1"/>
+      <c r="B15" s="9">
+        <f>1-B14/C29</f>
+        <v>0.96220220220220221</v>
+      </c>
+      <c r="C15" s="9">
+        <f>1-C14/C29</f>
+        <v>0.97431031031031035</v>
+      </c>
+      <c r="D15" s="9">
+        <f>1-D14/C29</f>
+        <v>0.9671564898231565</v>
+      </c>
+      <c r="E15" s="9">
+        <f>1-E14/C29</f>
+        <v>0.90123456790123457</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
-        <f aca="false">generated_image!A9</f>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A16" s="1">
+        <f>generated_image!A9</f>
         <v>100000000</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="8">
         <v>1330</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="8">
         <v>860</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="8">
         <v>1346</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="8">
         <v>3814</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11" t="n">
-        <f aca="false">1-B16/C29</f>
-        <v>0.985799132465799</v>
-      </c>
-      <c r="C17" s="11" t="n">
-        <f aca="false">1-C16/C29</f>
-        <v>0.990817484150818</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <f aca="false">1-D16/C29</f>
-        <v>0.985628294961628</v>
-      </c>
-      <c r="E17" s="11" t="n">
-        <f aca="false">1-E16/C29</f>
-        <v>0.959276609943277</v>
-      </c>
-      <c r="F17" s="9" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A17" s="1"/>
+      <c r="B17" s="9">
+        <f>1-B16/C29</f>
+        <v>0.98579913246579909</v>
+      </c>
+      <c r="C17" s="9">
+        <f>1-C16/C29</f>
+        <v>0.9908174841508175</v>
+      </c>
+      <c r="D17" s="9">
+        <f>1-D16/C29</f>
+        <v>0.98562829496162829</v>
+      </c>
+      <c r="E17" s="9">
+        <f>1-E16/C29</f>
+        <v>0.95927660994327657</v>
+      </c>
+      <c r="F17" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
-        <f aca="false">generated_image!A10</f>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A18" s="1">
+        <f>generated_image!A10</f>
         <v>50000000</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="8">
         <v>746</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="8">
         <v>286</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="8">
         <v>718</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="8">
         <v>3146</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F18" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11" t="n">
-        <f aca="false">1-B18/C29</f>
-        <v>0.992034701368035</v>
-      </c>
-      <c r="C19" s="11" t="n">
-        <f aca="false">1-C18/C29</f>
-        <v>0.996946279612946</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <f aca="false">1-D18/C29</f>
-        <v>0.992333667000334</v>
-      </c>
-      <c r="E19" s="11" t="n">
-        <f aca="false">1-E18/C29</f>
-        <v>0.966409075742409</v>
-      </c>
-      <c r="F19" s="9" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A19" s="1"/>
+      <c r="B19" s="9">
+        <f>1-B18/C29</f>
+        <v>0.99203470136803473</v>
+      </c>
+      <c r="C19" s="9">
+        <f>1-C18/C29</f>
+        <v>0.99694627961294624</v>
+      </c>
+      <c r="D19" s="9">
+        <f>1-D18/C29</f>
+        <v>0.99233366700033365</v>
+      </c>
+      <c r="E19" s="9">
+        <f>1-E18/C29</f>
+        <v>0.96640907574240908</v>
+      </c>
+      <c r="F19" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="1" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="B29" t="s">
         <v>5</v>
       </c>
-      <c r="C29" s="1" t="n">
-        <f aca="false">999*250*3/8</f>
+      <c r="C29">
+        <f>999*250*3/8</f>
         <v>93656.25</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A19"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>

</xml_diff>